<commit_message>
Project portal generator (self-contained HTML index + 3D viewer)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/06-wrapup/CFU-000-PM-REG-001_Document-Register.xlsx
+++ b/deliverables/06-wrapup/CFU-000-PM-REG-001_Document-Register.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -901,7 +901,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CFU-000-IC-CSD-006</t>
+          <t>CFU-000-IC-BLK-001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>BLK</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>APC MPC Structure</t>
+          <t>ICS Architecture</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -936,14 +936,14 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CFU-000-IC-IDX-001</t>
+          <t>CFU-000-IC-CAL-001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDX</t>
+          <t>CAL</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Instrument Index</t>
+          <t>Control Valve Sizing</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CFU-000-ME-CAL-001</t>
+          <t>CFU-000-IC-CE-001</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -995,17 +995,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CAL</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mechanical Design Calculations</t>
+          <t>Cause Effect Matrix</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1015,19 +1015,19 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>md, pdf</t>
+          <t>pdf, svg, xlsx</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-000</t>
+          <t>CFU-000-IC-CSD-006</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Equipment Datasheets Combined</t>
+          <t>APC MPC Structure</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1057,19 +1057,19 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-001</t>
+          <t>CFU-000-IC-CSD-ALL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1079,17 +1079,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Columns Datasheets</t>
+          <t>Control Scheme Diagrams</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1104,14 +1104,14 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-002</t>
+          <t>CFU-000-IC-IDX-001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1121,17 +1121,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>IDX</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Drums Desalters Datasheets</t>
+          <t>Instrument Index</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1141,19 +1141,19 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-003</t>
+          <t>CFU-000-IC-IOL-001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1163,17 +1163,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>IOL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fired Heaters Datasheets</t>
+          <t>IO List</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1183,19 +1183,19 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-004</t>
+          <t>CFU-000-IC-RPT-001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1205,17 +1205,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Shell Tube Exchangers Datasheets</t>
+          <t>Control Philosophy</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1225,19 +1225,19 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-005</t>
+          <t>CFU-000-IC-RPT-002</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1247,17 +1247,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Air Coolers Datasheets</t>
+          <t>SIF List SIL Determination</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1267,19 +1267,19 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>02-equipment</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-006</t>
+          <t>CFU-000-ME-CAL-001</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>CAL</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pumps Datasheets</t>
+          <t>Mechanical Design Calculations</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CFU-000-ME-DS-007</t>
+          <t>CFU-000-ME-DS-000</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pressure Relief Valves Datasheets</t>
+          <t>Equipment Datasheets Combined</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1363,7 +1363,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CFU-000-ME-LST-001</t>
+          <t>CFU-000-ME-DS-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1378,12 +1378,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LST</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Equipment List</t>
+          <t>Columns Datasheets</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1405,7 +1405,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CFU-000-PI-LL-001</t>
+          <t>CFU-000-ME-DS-002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1415,17 +1415,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Piping</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LL</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Line List</t>
+          <t>Drums Desalters Datasheets</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1435,19 +1435,19 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>03-layout-piping</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CFU-000-PI-SPC-001</t>
+          <t>CFU-000-ME-DS-003</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1457,17 +1457,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Piping</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SPC</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Piping Class Summary</t>
+          <t>Fired Heaters Datasheets</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1477,19 +1477,19 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>md, xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>03-layout-piping</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CFU-000-PL-3DM-001</t>
+          <t>CFU-000-ME-DS-004</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1499,17 +1499,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Plant layout</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3DM</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>render iso NE C101</t>
+          <t>Shell Tube Exchangers Datasheets</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1519,19 +1519,19 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>glb, png</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>03-layout-piping/3d</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CFU-000-PL-ELV-001</t>
+          <t>CFU-000-ME-DS-005</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1541,17 +1541,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Plant layout</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ELV</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Section C101 H101</t>
+          <t>Air Coolers Datasheets</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1561,19 +1561,19 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>03-layout-piping/layout</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CFU-000-PL-ELV-002</t>
+          <t>CFU-000-ME-DS-006</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1583,17 +1583,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Plant layout</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ELV</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Section C201 H201</t>
+          <t>Pumps Datasheets</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1603,19 +1603,19 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>03-layout-piping/layout</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CFU-000-PL-ELV-003</t>
+          <t>CFU-000-ME-DS-007</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1625,17 +1625,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Plant layout</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ELV</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pipe Rack Section</t>
+          <t>Pressure Relief Valves Datasheets</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1645,19 +1645,19 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>03-layout-piping/layout</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CFU-000-PL-PLT-001</t>
+          <t>CFU-000-ME-LST-001</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1667,17 +1667,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Plant layout</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PLT</t>
+          <t>LST</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Plot Plan</t>
+          <t>Equipment List</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1687,19 +1687,19 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>03-layout-piping/layout</t>
+          <t>02-equipment</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CFU-000-PM-EST-001</t>
+          <t>CFU-000-PI-LL-001</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1709,17 +1709,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Project management</t>
+          <t>Piping</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EST</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Cost Estimate</t>
+          <t>Line List</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>md, pdf, xlsx</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>06-wrapup</t>
+          <t>03-layout-piping</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CFU-000-PM-REG-001</t>
+          <t>CFU-000-PI-SPC-001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1751,17 +1751,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Project management</t>
+          <t>Piping</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>SPC</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Document Register</t>
+          <t>Piping Class Summary</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1771,19 +1771,19 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>md, pdf, xlsx</t>
+          <t>md, xlsx</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>06-wrapup</t>
+          <t>03-layout-piping</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CFU-000-PR-BFD-001</t>
+          <t>CFU-000-PL-3DM-001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1793,17 +1793,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Plant layout</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BFD</t>
+          <t>3DM</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>render iso NE C101</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1813,19 +1813,19 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>glb, png</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>01-process/bfd</t>
+          <t>03-layout-piping/3d</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CFU-000-PR-BOD-001</t>
+          <t>CFU-000-PL-ELV-001</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1835,17 +1835,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Plant layout</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>BOD</t>
+          <t>ELV</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Basis of Design</t>
+          <t>Section C101 H101</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1855,19 +1855,19 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>md, pdf</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>03-layout-piping/layout</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CFU-000-PR-HMB-001</t>
+          <t>CFU-000-PL-ELV-002</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1877,17 +1877,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Plant layout</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>HMB</t>
+          <t>ELV</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Heat Material Balance</t>
+          <t>Section C201 H201</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1897,19 +1897,19 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>03-layout-piping/layout</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PFD-ALL</t>
+          <t>CFU-000-PL-ELV-003</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1919,17 +1919,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Plant layout</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>ELV</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Pipe Rack Section</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1939,19 +1939,19 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>03-layout-piping/layout</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PID-000</t>
+          <t>CFU-000-PL-PLT-001</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Plant layout</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PLT</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Plot Plan</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1986,14 +1986,14 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>03-layout-piping/layout</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PID-ALL</t>
+          <t>CFU-000-PM-EST-001</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Project management</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>EST</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Cost Estimate</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2023,19 +2023,19 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CFU-000-PR-RPT-001</t>
+          <t>CFU-000-PM-REG-001</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2045,17 +2045,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Project management</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RPT</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Process Design Report</t>
+          <t>Document Register</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2065,19 +2065,19 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>md, pdf</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CFU-000-PR-RPT-002</t>
+          <t>CFU-000-PR-BFD-001</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RPT</t>
+          <t>BFD</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Preliminary HAZOP</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2107,39 +2107,39 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>md, pdf, xlsx</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>06-wrapup</t>
+          <t>01-process/bfd</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-001</t>
+          <t>CFU-000-PR-BOD-001</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>BOD</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>H 101 Combustion Control</t>
+          <t>Basis of Design</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2149,39 +2149,39 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-002</t>
+          <t>CFU-000-PR-HMB-001</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>HMB</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>C 101 Column Control</t>
+          <t>Heat Material Balance</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2191,39 +2191,39 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-003</t>
+          <t>CFU-000-PR-PFD-ALL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Desalting Preheat Control</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2233,39 +2233,39 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-004</t>
+          <t>CFU-000-PR-PID-000</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Stabiliser Splitter Control</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2280,34 +2280,34 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-001</t>
+          <t>CFU-000-PR-PID-ALL</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>C 101 Column GA</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2317,39 +2317,39 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-002</t>
+          <t>CFU-000-PR-RPT-001</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Side Strippers GA</t>
+          <t>Process Design Report</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2359,39 +2359,39 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-003</t>
+          <t>CFU-000-PR-RPT-002</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>C 105 C 106 GA</t>
+          <t>Preliminary HAZOP</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2401,19 +2401,19 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-005</t>
+          <t>CFU-100-IC-CSD-001</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2423,17 +2423,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>H 101 Heater GA</t>
+          <t>H 101 Combustion Control</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2448,14 +2448,14 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-007</t>
+          <t>CFU-100-IC-CSD-002</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2465,17 +2465,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>D 101AB Desalter GA</t>
+          <t>C 101 Column Control</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2490,14 +2490,14 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-008</t>
+          <t>CFU-100-IC-CSD-003</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>AES Exchanger Setting Plan</t>
+          <t>Desalting Preheat Control</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2532,14 +2532,14 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-001</t>
+          <t>CFU-100-IC-CSD-004</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2549,17 +2549,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Stabiliser Splitter Control</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2574,14 +2574,14 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-002</t>
+          <t>CFU-100-IC-LD-001</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2591,17 +2591,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>FIC 1031</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2616,14 +2616,14 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>04-instrumentation/loop-diagrams</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-003</t>
+          <t>CFU-100-IC-LD-002</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2633,17 +2633,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>TIC 1020 PIC 1021</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2658,14 +2658,14 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>04-instrumentation/loop-diagrams</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-004</t>
+          <t>CFU-100-IC-LD-003</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2675,17 +2675,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>SIF 101</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2700,14 +2700,14 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>04-instrumentation/loop-diagrams</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-001</t>
+          <t>CFU-100-IC-LD-ALL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2717,17 +2717,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Loop Diagrams</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2737,19 +2737,19 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-002</t>
+          <t>CFU-100-ME-GA-001</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2759,17 +2759,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>C 101 Column GA</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2784,14 +2784,14 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-003</t>
+          <t>CFU-100-ME-GA-002</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Side Strippers GA</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2826,14 +2826,14 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-004</t>
+          <t>CFU-100-ME-GA-003</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2843,17 +2843,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>C 105 C 106 GA</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2868,14 +2868,14 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-005</t>
+          <t>CFU-100-ME-GA-005</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2885,17 +2885,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>H 101 Heater GA</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2910,14 +2910,14 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-006</t>
+          <t>CFU-100-ME-GA-007</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2927,17 +2927,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>D 101AB Desalter GA</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2952,14 +2952,14 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-007</t>
+          <t>CFU-100-ME-GA-008</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2969,17 +2969,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>AES Exchanger Setting Plan</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2994,14 +2994,14 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-008</t>
+          <t>CFU-100-PR-PFD-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3036,14 +3036,14 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-009</t>
+          <t>CFU-100-PR-PFD-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3078,14 +3078,14 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-010</t>
+          <t>CFU-100-PR-PFD-003</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3120,14 +3120,14 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-011</t>
+          <t>CFU-100-PR-PFD-004</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3162,34 +3162,34 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CFU-200-IC-CSD-005</t>
+          <t>CFU-100-PR-PID-001</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>VDU Control</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3204,34 +3204,34 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CFU-200-ME-GA-004</t>
+          <t>CFU-100-PR-PID-002</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>C 201 Vacuum Column GA</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3246,34 +3246,34 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CFU-200-ME-GA-006</t>
+          <t>CFU-100-PR-PID-003</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>H 201 Heater GA</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3288,19 +3288,19 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PFD-005</t>
+          <t>CFU-100-PR-PID-004</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3330,19 +3330,19 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PFD-006</t>
+          <t>CFU-100-PR-PID-005</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3372,19 +3372,19 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-012</t>
+          <t>CFU-100-PR-PID-006</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3421,12 +3421,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-013</t>
+          <t>CFU-100-PR-PID-007</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3463,12 +3463,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-014</t>
+          <t>CFU-100-PR-PID-008</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3505,12 +3505,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-015</t>
+          <t>CFU-100-PR-PID-009</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3547,40 +3547,502 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>CFU-100-PR-PID-010</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CFU-100-PR-PID-011</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CFU-200-IC-CSD-005</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Instrumentation &amp; control</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>CSD</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>VDU Control</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>04-instrumentation/control-scheme</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>CFU-200-ME-GA-004</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>C 201 Vacuum Column GA</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>02-equipment/ga</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>CFU-200-ME-GA-006</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>H 201 Heater GA</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>02-equipment/ga</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PFD-005</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>01-process/pfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PFD-006</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>PFD</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>01-process/pfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PID-012</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PID-013</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PID-014</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PID-015</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>CFU-900-PR-PID-016</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>PID</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>(drawing)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>pdf, svg</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>01-process/pid</t>
         </is>

</xml_diff>

<commit_message>
Add design dependency map checked against the build
Activity network of 45 design steps (issued and still to do) with inputs,
external inputs, owned data, deliverables and 15 iteration loops. Generates
CFU-000-PM-DEP-001 (report + workbook with DSM, change impact, to-do list),
CFU-000-PM-DEP-002 (network drawing) and an interactive portal page.

A traced build (python -m cfu.wrapup.depmap --trace) records which module
reads which data file; all 62 reads are covered by the map. The trace showed
the P&ID stage read layout.json before the layout stage wrote it, so layout
now runs before pid in build.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/06-wrapup/CFU-000-PM-REG-001_Document-Register.xlsx
+++ b/deliverables/06-wrapup/CFU-000-PM-REG-001_Document-Register.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2161,7 +2161,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CFU-000-PM-EST-001</t>
+          <t>CFU-000-PM-DEP-001</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EST</t>
+          <t>DEP</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Cost Estimate</t>
+          <t>Design Dependency Map</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2203,7 +2203,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CFU-000-PM-REG-001</t>
+          <t>CFU-000-PM-DEP-002</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2218,12 +2218,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>DEP</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Document Register</t>
+          <t>Design Network Diagram</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>md, pdf, xlsx</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2245,7 +2245,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CFU-000-PR-BFD-001</t>
+          <t>CFU-000-PM-EST-001</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2255,17 +2255,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Project management</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BFD</t>
+          <t>EST</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Cost Estimate</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2275,19 +2275,19 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>01-process/bfd</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CFU-000-PR-BOD-001</t>
+          <t>CFU-000-PM-REG-001</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2297,17 +2297,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Project management</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BOD</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Basis of Design</t>
+          <t>Document Register</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2317,19 +2317,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>md, pdf</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CFU-000-PR-HMB-001</t>
+          <t>CFU-000-PR-BFD-001</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>HMB</t>
+          <t>BFD</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Heat Material Balance</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2359,19 +2359,19 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>01-process/bfd</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PFD-ALL</t>
+          <t>CFU-000-PR-BOD-001</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2386,12 +2386,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>BOD</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Basis of Design</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2401,19 +2401,19 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PID-000</t>
+          <t>CFU-000-PR-HMB-001</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>HMB</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Heat Material Balance</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2443,19 +2443,19 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>xlsx</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CFU-000-PR-PID-ALL</t>
+          <t>CFU-000-PR-PFD-ALL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2490,14 +2490,14 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CFU-000-PR-RPT-001</t>
+          <t>CFU-000-PR-PID-000</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2512,12 +2512,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>RPT</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Process Design Report</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2527,19 +2527,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>md, pdf</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>00-basis</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CFU-000-PR-RPT-002</t>
+          <t>CFU-000-PR-PID-ALL</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2554,12 +2554,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>RPT</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Preliminary HAZOP</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2569,39 +2569,39 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>md, pdf, xlsx</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>06-wrapup</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-001</t>
+          <t>CFU-000-PR-RPT-001</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>H 101 Combustion Control</t>
+          <t>Process Design Report</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2611,39 +2611,39 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>00-basis</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-002</t>
+          <t>CFU-000-PR-RPT-002</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>000</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>RPT</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>C 101 Column Control</t>
+          <t>Preliminary HAZOP</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2653,19 +2653,19 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>md, pdf, xlsx</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>06-wrapup</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-003</t>
+          <t>CFU-100-IC-CSD-001</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Desalting Preheat Control</t>
+          <t>H 101 Combustion Control</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2707,7 +2707,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CFU-100-IC-CSD-004</t>
+          <t>CFU-100-IC-CSD-002</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Stabiliser Splitter Control</t>
+          <t>C 101 Column Control</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2749,7 +2749,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CFU-100-IC-LD-001</t>
+          <t>CFU-100-IC-CSD-003</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2764,12 +2764,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>LD</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FIC 1031</t>
+          <t>Desalting Preheat Control</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2784,14 +2784,14 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>04-instrumentation/loop-diagrams</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CFU-100-IC-LD-002</t>
+          <t>CFU-100-IC-CSD-004</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2806,12 +2806,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>LD</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>TIC 1020 PIC 1021</t>
+          <t>Stabiliser Splitter Control</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2826,14 +2826,14 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>04-instrumentation/loop-diagrams</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CFU-100-IC-LD-003</t>
+          <t>CFU-100-IC-LD-001</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SIF 101</t>
+          <t>FIC 1031</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CFU-100-IC-LD-ALL</t>
+          <t>CFU-100-IC-LD-002</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Loop Diagrams</t>
+          <t>TIC 1020 PIC 1021</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2905,19 +2905,19 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pdf, svg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>04-instrumentation</t>
+          <t>04-instrumentation/loop-diagrams</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-001</t>
+          <t>CFU-100-IC-LD-003</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2927,17 +2927,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>C 101 Column GA</t>
+          <t>SIF 101</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2952,14 +2952,14 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation/loop-diagrams</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-002</t>
+          <t>CFU-100-IC-LD-ALL</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2969,17 +2969,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>LD</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Side Strippers GA</t>
+          <t>Loop Diagrams</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2989,19 +2989,19 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>pdf, svg</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-003</t>
+          <t>CFU-100-ME-GA-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>C 105 C 106 GA</t>
+          <t>C 101 Column GA</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3043,7 +3043,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-005</t>
+          <t>CFU-100-ME-GA-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>H 101 Heater GA</t>
+          <t>Side Strippers GA</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3085,7 +3085,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-007</t>
+          <t>CFU-100-ME-GA-003</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>D 101AB Desalter GA</t>
+          <t>C 105 C 106 GA</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3127,7 +3127,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CFU-100-ME-GA-008</t>
+          <t>CFU-100-ME-GA-005</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AES Exchanger Setting Plan</t>
+          <t>H 101 Heater GA</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3169,7 +3169,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-001</t>
+          <t>CFU-100-ME-GA-007</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3179,17 +3179,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Piping</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ISO</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>H 101 Outlet Transfer Line To C 101</t>
+          <t>D 101AB Desalter GA</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3204,14 +3204,14 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>03-layout-piping/piping/iso</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-002</t>
+          <t>CFU-100-ME-GA-008</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3221,17 +3221,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Piping</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ISO</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>C 101 Overhead Vapour To A 101</t>
+          <t>AES Exchanger Setting Plan</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3246,14 +3246,14 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>03-layout-piping/piping/iso</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-003</t>
+          <t>CFU-100-PI-ISO-001</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>C 101 Bottoms To P 112A B Suction</t>
+          <t>H 101 Outlet Transfer Line To C 101</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3295,7 +3295,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-004</t>
+          <t>CFU-100-PI-ISO-002</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>P 112A B Discharge To H 201 Inlet SH1</t>
+          <t>C 101 Overhead Vapour To A 101</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-005</t>
+          <t>CFU-100-PI-ISO-003</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Crude Suction To P 101A B</t>
+          <t>C 101 Bottoms To P 112A B Suction</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3379,7 +3379,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-006</t>
+          <t>CFU-100-PI-ISO-004</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>P 101A B Discharge To E 101</t>
+          <t>P 112A B Discharge To H 201 Inlet SH1</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3421,7 +3421,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-007</t>
+          <t>CFU-100-PI-ISO-005</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>C 101 Bpa Draw To P 108A B</t>
+          <t>Crude Suction To P 101A B</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-008</t>
+          <t>CFU-100-PI-ISO-006</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Bpa Return E 113 To C 101</t>
+          <t>P 101A B Discharge To E 101</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3505,7 +3505,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-009</t>
+          <t>CFU-100-PI-ISO-007</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>C 101 Kero Draw To C 102 Gravity</t>
+          <t>C 101 Bpa Draw To P 108A B</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3547,7 +3547,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-010</t>
+          <t>CFU-100-PI-ISO-008</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>D 102 To P 103A B Suction</t>
+          <t>Bpa Return E 113 To C 101</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3589,7 +3589,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-011</t>
+          <t>CFU-100-PI-ISO-009</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>D 102 To P 104A B Suction</t>
+          <t>C 101 Kero Draw To C 102 Gravity</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3631,7 +3631,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CFU-100-PI-ISO-012</t>
+          <t>CFU-100-PI-ISO-010</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Hp Steam Header To E 116</t>
+          <t>D 102 To P 103A B Suction</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3673,7 +3673,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-001</t>
+          <t>CFU-100-PI-ISO-011</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3683,17 +3683,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Piping</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>ISO</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>D 102 To P 104A B Suction</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3708,14 +3708,14 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>03-layout-piping/piping/iso</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-002</t>
+          <t>CFU-100-PI-ISO-012</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3725,17 +3725,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Piping</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>ISO</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>Hp Steam Header To E 116</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3750,14 +3750,14 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>03-layout-piping/piping/iso</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-003</t>
+          <t>CFU-100-PR-PFD-001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3799,7 +3799,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PFD-004</t>
+          <t>CFU-100-PR-PFD-002</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3841,7 +3841,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-001</t>
+          <t>CFU-100-PR-PFD-003</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3876,14 +3876,14 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-002</t>
+          <t>CFU-100-PR-PFD-004</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3918,14 +3918,14 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-003</t>
+          <t>CFU-100-PR-PID-001</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3967,7 +3967,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-004</t>
+          <t>CFU-100-PR-PID-002</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4009,7 +4009,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-005</t>
+          <t>CFU-100-PR-PID-003</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4051,7 +4051,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-006</t>
+          <t>CFU-100-PR-PID-004</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4093,7 +4093,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-007</t>
+          <t>CFU-100-PR-PID-005</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4135,7 +4135,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-008</t>
+          <t>CFU-100-PR-PID-006</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4177,7 +4177,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-009</t>
+          <t>CFU-100-PR-PID-007</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4219,7 +4219,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-010</t>
+          <t>CFU-100-PR-PID-008</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4261,7 +4261,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CFU-100-PR-PID-011</t>
+          <t>CFU-100-PR-PID-009</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4303,27 +4303,27 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CFU-200-IC-CSD-005</t>
+          <t>CFU-100-PR-PID-010</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Instrumentation &amp; control</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>CSD</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>VDU Control</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4338,34 +4338,34 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>04-instrumentation/control-scheme</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CFU-200-ME-GA-004</t>
+          <t>CFU-100-PR-PID-011</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>PID</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>C 201 Vacuum Column GA</t>
+          <t>(drawing)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4380,14 +4380,14 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>01-process/pid</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CFU-200-ME-GA-006</t>
+          <t>CFU-200-IC-CSD-005</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4397,17 +4397,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>Instrumentation &amp; control</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>CSD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>H 201 Heater GA</t>
+          <t>VDU Control</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4422,14 +4422,14 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>02-equipment/ga</t>
+          <t>04-instrumentation/control-scheme</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CFU-200-PI-ISO-001</t>
+          <t>CFU-200-ME-GA-004</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4439,17 +4439,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Piping</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>ISO</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>H 201 Outlet Vacuum Transfer Line To C 201</t>
+          <t>C 201 Vacuum Column GA</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4464,14 +4464,14 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>03-layout-piping/piping/iso</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PFD-005</t>
+          <t>CFU-200-ME-GA-006</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4481,17 +4481,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>H 201 Heater GA</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4506,14 +4506,14 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>02-equipment/ga</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PFD-006</t>
+          <t>CFU-200-PI-ISO-001</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Piping</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PFD</t>
+          <t>ISO</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>(drawing)</t>
+          <t>H 201 Outlet Vacuum Transfer Line To C 201</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4548,14 +4548,14 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>01-process/pfd</t>
+          <t>03-layout-piping/piping/iso</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-012</t>
+          <t>CFU-200-PR-PFD-005</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4590,14 +4590,14 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-013</t>
+          <t>CFU-200-PR-PFD-006</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>PID</t>
+          <t>PFD</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4632,14 +4632,14 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>01-process/pid</t>
+          <t>01-process/pfd</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-014</t>
+          <t>CFU-200-PR-PID-012</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4681,7 +4681,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CFU-200-PR-PID-015</t>
+          <t>CFU-200-PR-PID-013</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4723,40 +4723,124 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>CFU-200-PR-PID-014</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>CFU-200-PR-PID-015</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>PID</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>(drawing)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>01-process/pid</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
           <t>CFU-900-PR-PID-016</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D105" t="inlineStr">
         <is>
           <t>PID</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>(drawing)</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>pdf, svg</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>pdf, svg</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
         <is>
           <t>01-process/pid</t>
         </is>

</xml_diff>